<commit_message>
Migrate the lupin.com footer and add the Lupin logo to the nav
- footer: lead column (address, contacts, LinkedIn), three link columns and
  copyright bar built from the footer fragment; hover underline/fade, back to
  top, "#_blank" new-tab marker, decorative flower and chevron block assets;
  desktop values in vw from the source at 1440px, mobile-first stack at 375px
- header: size the brand logo like the source (91px at 375px, 101px at 1440px)
- fonts: Helvetica Neue Medium from lupin.com
- importer: footer import and nav import (logo from the source header)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="45">
   <si>
     <t>_reportFile</t>
   </si>
@@ -22,9 +22,15 @@
     <t>links</t>
   </si>
   <si>
+    <t>logo</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
+    <t>sections</t>
+  </si>
+  <si>
     <t>status</t>
   </si>
   <si>
@@ -40,43 +46,106 @@
     <t>url</t>
   </si>
   <si>
+    <t>footer.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>footer</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-10-05T19:22:48.909Z</t>
+  </si>
+  <si>
+    <t>https://www.lupin.com/US/product</t>
+  </si>
+  <si>
     <t>nav.report.json</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>["Contact your Representative"]</t>
+    <t>["Contact Your Representative"]</t>
+  </si>
+  <si>
+    <t>https://www.lupin.com/US/images/lupin_logo.webp</t>
   </si>
   <si>
     <t>nav</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>2026-10-05T10:32:51.268Z</t>
-  </si>
-  <si>
-    <t>https://www.lupin.com/US/product</t>
+    <t>2026-10-06T02:12:30.265Z</t>
+  </si>
+  <si>
+    <t>us/contact-us.report.json</t>
+  </si>
+  <si>
+    <t>["hero-map","cards-location","form-contact","columns-contacts"]</t>
+  </si>
+  <si>
+    <t>us/contact-us</t>
+  </si>
+  <si>
+    <t>contact-us</t>
+  </si>
+  <si>
+    <t>2026-10-05T14:56:25.891Z</t>
+  </si>
+  <si>
+    <t>Contact Lupin US | Get in Touch with Our Team</t>
+  </si>
+  <si>
+    <t>https://www.lupin.com/US/contact-us</t>
+  </si>
+  <si>
+    <t>us/hcpportal.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-product","cards-link-tile","cards-link-tile"]</t>
+  </si>
+  <si>
+    <t>us/hcpportal</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>2026-10-05T18:14:40.021Z</t>
+  </si>
+  <si>
+    <t>Explore Our Products | Quality Medicines for Better Health.</t>
   </si>
   <si>
     <t>us/product.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","cards-product","cards-link-tile","cards-link-tile"]</t>
-  </si>
-  <si>
     <t>us/product</t>
   </si>
   <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>2026-10-05T10:28:00.088Z</t>
-  </si>
-  <si>
-    <t>Explore Our Products | Quality Medicines for Better Health.</t>
+    <t>2026-10-05T14:55:04.507Z</t>
+  </si>
+  <si>
+    <t>us/product/glycerol-phenylbutyrate-oral-liquid.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-product-detail","tabs-audience","columns-anchor-nav","columns-anchor-nav","hero-green-panel","hero-green-panel","columns-icon-tips","cards-pharmacy","cards-pharmacy","accordion-faq","accordion-faq","columns-cta-banner","columns-cta-banner"]</t>
+  </si>
+  <si>
+    <t>us/product/glycerol-phenylbutyrate-oral-liquid</t>
+  </si>
+  <si>
+    <t>product-detail</t>
+  </si>
+  <si>
+    <t>2026-10-05T17:10:00.610Z</t>
+  </si>
+  <si>
+    <t>Glycerol Phenylbutyrate Oral Liquid</t>
+  </si>
+  <si>
+    <t>https://www.lupin.com/US/product/glycerol-phenylbutyrate-oral-liquid</t>
   </si>
 </sst>
 </file>
@@ -465,20 +534,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="4" max="4" width="49" customWidth="1"/>
+    <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,16 +575,22 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -523,50 +598,202 @@
       <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
-        <v>12</v>
+      <c r="F2">
+        <v>5</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
       </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" t="s">
+        <v>43</v>
+      </c>
+      <c r="K7" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a Register link with a registration dialog to the nav
Links to #register open a dialog asking for first name, last name and email;
"Register Now" validates the fields and stores them in the lupin_registration
cookie (JSON, one year, Path=/, SameSite=Lax, Secure on https). The dialog
lives in scripts/register.js and is wired up by the header block.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -67,7 +67,7 @@
     <t>nav.report.json</t>
   </si>
   <si>
-    <t>["Contact Your Representative"]</t>
+    <t>["Contact Your Representative","Register"]</t>
   </si>
   <si>
     <t>https://www.lupin.com/US/images/lupin_logo.webp</t>
@@ -76,7 +76,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-10-06T02:12:30.265Z</t>
+    <t>2026-10-06T09:05:00.957Z</t>
   </si>
   <si>
     <t>us/contact-us.report.json</t>
@@ -538,7 +538,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="49" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>

</xml_diff>

<commit_message>
Add a Sign out link to the nav that clears the registration cookie
Links to /sign-out delete lupin_registration and fire REGISTRATION_EVENT
with null, which removes the nav greeting and the Marketo name values
that were pre-filled. The link only shows while someone is registered.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -67,7 +67,7 @@
     <t>nav.report.json</t>
   </si>
   <si>
-    <t>["Contact Your Representative","Register"]</t>
+    <t>["Contact Your Representative","Register","Sign out"]</t>
   </si>
   <si>
     <t>https://www.lupin.com/US/images/lupin_logo.webp</t>
@@ -76,7 +76,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-10-06T10:01:52.119Z</t>
+    <t>2026-10-06T13:42:12.567Z</t>
   </si>
   <si>
     <t>us/contact-us.report.json</t>
@@ -537,8 +537,7 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="4" max="4" width="49" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>

</xml_diff>

<commit_message>
Nav import: use the uploaded logo and the Register/Sign In label
The importer now matches the nav authored in Document Authoring, so a
content sync from the workspace keeps the uploaded logo and label.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-nav.report.xlsx
+++ b/tools/importer/reports/import-nav.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="53">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>links</t>
   </si>
   <si>
@@ -67,16 +73,40 @@
     <t>nav.report.json</t>
   </si>
   <si>
-    <t>["Contact Your Representative","Register","Sign out"]</t>
-  </si>
-  <si>
-    <t>https://www.lupin.com/US/images/lupin_logo.webp</t>
+    <t>["Contact Your Representative","Register/Sign In","Sign out"]</t>
+  </si>
+  <si>
+    <t>https://main--lupinus--cpanditadobe.aem.live/media_1fbb4975e5a28eac21c41458115f499d47b8b6bb2.png</t>
   </si>
   <si>
     <t>nav</t>
   </si>
   <si>
-    <t>2026-10-06T13:42:12.567Z</t>
+    <t>2026-10-06T16:03:36.330Z</t>
+  </si>
+  <si>
+    <t>US/product.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: logo is not defined
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: logo is not defined
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:693:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:956:22)</t>
+  </si>
+  <si>
+    <t>US/product</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-10-06T16:03:10.506Z</t>
   </si>
   <si>
     <t>us/contact-us.report.json</t>
@@ -534,19 +564,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="49" customWidth="1"/>
-    <col min="5" max="5" width="48" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="11" width="50" customWidth="1"/>
+    <col min="1" max="6" width="50" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="26" customWidth="1"/>
+    <col min="12" max="13" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -580,219 +609,302 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2">
         <v>5</v>
       </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
       <c r="I2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
-        <v>12</v>
-      </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="J3" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="K3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
         <v>16</v>
       </c>
+      <c r="J5" t="s">
+        <v>33</v>
+      </c>
+      <c r="K5" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" t="s">
-        <v>28</v>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" t="s">
+        <v>40</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K5" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" t="s">
         <v>16</v>
       </c>
+      <c r="J7" t="s">
+        <v>40</v>
+      </c>
+      <c r="K7" t="s">
+        <v>45</v>
+      </c>
+      <c r="L7" t="s">
+        <v>42</v>
+      </c>
+      <c r="M7" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K6" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" t="s">
-        <v>42</v>
-      </c>
-      <c r="J7" t="s">
-        <v>43</v>
-      </c>
-      <c r="K7" t="s">
-        <v>44</v>
+      <c r="J8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" t="s">
+        <v>50</v>
+      </c>
+      <c r="L8" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>